<commit_message>
Major updates: Mobile responsiveness, map chart improvements, and comprehensive README
- Mobile responsive design: Timeline chart optimized for mobile with responsive margins, fonts, and layouts
- Map chart improvements: Show cities and work experiences (exclude education) with better tooltips
- Timeline legend: Positioned optimally for desktop and mobile, single-line layout
- Comprehensive README: Beautiful storytelling with technical details, architecture, and deployment guides
- Mobile testing guide: Added MOBILE_TESTING.md with Chrome DevTools and real device testing instructions
- Memory optimizations: Maintained efficient memory usage for cloud deployment
</commit_message>
<xml_diff>
--- a/resume_data/resume_data.xlsx
+++ b/resume_data/resume_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="96">
   <si>
     <t>candidate_id</t>
   </si>
@@ -194,9 +194,6 @@
   </si>
   <si>
     <t>Senior Business Analyst</t>
-  </si>
-  <si>
-    <t>Employement</t>
   </si>
   <si>
     <t>Amazon</t>
@@ -1071,10 +1068,10 @@
         <v>1234.0</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>61</v>
       </c>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
@@ -1082,7 +1079,7 @@
         <v>59</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I11" s="1" t="s">
         <v>48</v>
@@ -1120,22 +1117,22 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="2">
@@ -1146,10 +1143,10 @@
         <v>1234.0</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>69</v>
       </c>
       <c r="E2" s="1">
         <v>2017.0</v>
@@ -1167,10 +1164,10 @@
         <v>1234.0</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E3" s="1">
         <v>2017.0</v>
@@ -1188,10 +1185,10 @@
         <v>1234.0</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>71</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="E4" s="1">
         <v>2012.0</v>
@@ -1209,10 +1206,10 @@
         <v>1234.0</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>73</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>74</v>
       </c>
       <c r="E5" s="1">
         <v>2021.0</v>
@@ -1230,10 +1227,10 @@
         <v>1234.0</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>75</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>76</v>
       </c>
       <c r="E6" s="1">
         <v>2021.0</v>
@@ -1251,10 +1248,10 @@
         <v>1234.0</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E7" s="1">
         <v>2017.0</v>
@@ -1272,10 +1269,10 @@
         <v>1234.0</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E8" s="1">
         <v>2017.0</v>
@@ -1293,10 +1290,10 @@
         <v>1234.0</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>80</v>
       </c>
       <c r="E9" s="1">
         <v>2018.0</v>
@@ -1314,10 +1311,10 @@
         <v>1234.0</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E10" s="1">
         <v>2023.0</v>
@@ -1335,10 +1332,10 @@
         <v>1234.0</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E11" s="1">
         <v>2012.0</v>
@@ -1356,10 +1353,10 @@
         <v>1234.0</v>
       </c>
       <c r="C12" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>83</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>84</v>
       </c>
       <c r="E12" s="1">
         <v>2012.0</v>
@@ -1377,10 +1374,10 @@
         <v>1234.0</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E13" s="1">
         <v>2012.0</v>
@@ -1398,10 +1395,10 @@
         <v>1234.0</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E14" s="1">
         <v>2017.0</v>
@@ -1419,10 +1416,10 @@
         <v>1234.0</v>
       </c>
       <c r="C15" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>87</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>88</v>
       </c>
       <c r="E15" s="1">
         <v>2024.0</v>
@@ -1440,10 +1437,10 @@
         <v>1234.0</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E16" s="1">
         <v>2017.0</v>
@@ -1461,10 +1458,10 @@
         <v>1234.0</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E17" s="1">
         <v>2017.0</v>
@@ -1482,10 +1479,10 @@
         <v>1234.0</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E18" s="1">
         <v>2018.0</v>
@@ -1503,10 +1500,10 @@
         <v>1234.0</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E19" s="1">
         <v>2018.0</v>
@@ -1524,10 +1521,10 @@
         <v>1234.0</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E20" s="1">
         <v>2018.0</v>
@@ -1545,10 +1542,10 @@
         <v>1234.0</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E21" s="1">
         <v>2018.0</v>
@@ -1566,10 +1563,10 @@
         <v>1234.0</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E22" s="1">
         <v>2012.0</v>
@@ -1587,10 +1584,10 @@
         <v>1234.0</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E23" s="1">
         <v>2024.0</v>
@@ -1617,7 +1614,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>15</v>

</xml_diff>

<commit_message>
Fix LinkedIn link and enable dynamic Excel data reloading
- Add format_url() function to ensure URLs have proper https:// protocol
- Implement dynamic data reloading from Excel on startup and dashboard access
- Fix LinkedIn link generation with proper URL formatting
- Add rel='noopener noreferrer' for security
- Update resume_data.xlsx with latest data
</commit_message>
<xml_diff>
--- a/resume_data/resume_data.xlsx
+++ b/resume_data/resume_data.xlsx
@@ -55,7 +55,7 @@
     <t>priyank.patil3@gmail.com</t>
   </si>
   <si>
-    <t>www.linkedin.com/in/priyank-patil</t>
+    <t>https://www.linkedin.com/in/priyank-patil</t>
   </si>
   <si>
     <t>https://github.com/priyankpatil</t>
@@ -311,7 +311,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -322,10 +322,6 @@
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <color rgb="FF0000FF"/>
     </font>
     <font>
       <u/>
@@ -350,7 +346,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -358,9 +354,6 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
@@ -371,7 +364,7 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -655,7 +648,7 @@
       <c r="G2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="2" t="s">
         <v>14</v>
       </c>
     </row>
@@ -725,7 +718,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4">
+      <c r="A2" s="3">
         <v>98745.0</v>
       </c>
       <c r="B2" s="1">
@@ -755,10 +748,10 @@
       <c r="J2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="K2" s="5">
+      <c r="K2" s="4">
         <v>39692.0</v>
       </c>
-      <c r="L2" s="5">
+      <c r="L2" s="4">
         <v>41061.0</v>
       </c>
       <c r="M2" s="1" t="b">
@@ -766,7 +759,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6">
+      <c r="A3" s="5">
         <v>98746.0</v>
       </c>
       <c r="B3" s="1">
@@ -792,10 +785,10 @@
       <c r="J3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="K3" s="5">
+      <c r="K3" s="4">
         <v>41141.0</v>
       </c>
-      <c r="L3" s="5">
+      <c r="L3" s="4">
         <v>42571.0</v>
       </c>
       <c r="M3" s="1" t="b">
@@ -803,7 +796,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6">
+      <c r="A4" s="5">
         <v>98747.0</v>
       </c>
       <c r="B4" s="1">
@@ -812,7 +805,7 @@
       <c r="C4" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="6" t="s">
         <v>38</v>
       </c>
       <c r="E4" s="1"/>
@@ -829,10 +822,10 @@
       <c r="J4" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="K4" s="5">
+      <c r="K4" s="4">
         <v>41537.0</v>
       </c>
-      <c r="L4" s="5">
+      <c r="L4" s="4">
         <v>41628.0</v>
       </c>
       <c r="M4" s="1" t="b">
@@ -840,7 +833,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6">
+      <c r="A5" s="5">
         <v>98748.0</v>
       </c>
       <c r="B5" s="1">
@@ -849,7 +842,7 @@
       <c r="C5" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>42</v>
       </c>
       <c r="E5" s="1"/>
@@ -866,10 +859,10 @@
       <c r="J5" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="K5" s="5">
+      <c r="K5" s="4">
         <v>41640.0</v>
       </c>
-      <c r="L5" s="5">
+      <c r="L5" s="4">
         <v>41944.0</v>
       </c>
       <c r="M5" s="1" t="b">
@@ -877,7 +870,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6">
+      <c r="A6" s="5">
         <v>98749.0</v>
       </c>
       <c r="B6" s="1">
@@ -907,10 +900,10 @@
       <c r="J6" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="K6" s="5">
+      <c r="K6" s="4">
         <v>42607.0</v>
       </c>
-      <c r="L6" s="5">
+      <c r="L6" s="4">
         <v>43229.0</v>
       </c>
       <c r="M6" s="1" t="b">
@@ -918,7 +911,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6">
+      <c r="A7" s="5">
         <v>98750.0</v>
       </c>
       <c r="B7" s="1">
@@ -944,10 +937,10 @@
       <c r="J7" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="K7" s="5">
+      <c r="K7" s="4">
         <v>42865.0</v>
       </c>
-      <c r="L7" s="5">
+      <c r="L7" s="4">
         <v>42962.0</v>
       </c>
       <c r="M7" s="1" t="b">
@@ -955,7 +948,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6">
+      <c r="A8" s="5">
         <v>98751.0</v>
       </c>
       <c r="B8" s="1">
@@ -981,10 +974,10 @@
       <c r="J8" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="K8" s="5">
+      <c r="K8" s="4">
         <v>43230.0</v>
       </c>
-      <c r="L8" s="5">
+      <c r="L8" s="4">
         <v>44397.0</v>
       </c>
       <c r="M8" s="1" t="b">
@@ -992,7 +985,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6">
+      <c r="A9" s="5">
         <v>98752.0</v>
       </c>
       <c r="B9" s="1">
@@ -1018,10 +1011,10 @@
       <c r="J9" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="K9" s="5">
+      <c r="K9" s="4">
         <v>44398.0</v>
       </c>
-      <c r="L9" s="5">
+      <c r="L9" s="4">
         <v>45005.0</v>
       </c>
       <c r="M9" s="1" t="b">
@@ -1029,7 +1022,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6">
+      <c r="A10" s="5">
         <v>98753.0</v>
       </c>
       <c r="B10" s="1">
@@ -1050,10 +1043,10 @@
       <c r="J10" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="K10" s="5">
+      <c r="K10" s="4">
         <v>45006.0</v>
       </c>
-      <c r="L10" s="5">
+      <c r="L10" s="4">
         <v>45903.0</v>
       </c>
       <c r="M10" s="1" t="b">
@@ -1061,7 +1054,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6">
+      <c r="A11" s="5">
         <v>98754.0</v>
       </c>
       <c r="B11" s="1">
@@ -1087,7 +1080,7 @@
       <c r="J11" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="K11" s="5">
+      <c r="K11" s="4">
         <v>45904.0</v>
       </c>
       <c r="M11" s="1" t="b">
@@ -1151,7 +1144,7 @@
       <c r="E2" s="1">
         <v>2017.0</v>
       </c>
-      <c r="F2" s="6">
+      <c r="F2" s="5">
         <f t="shared" ref="F2:F23" si="1">year(TODAY())-E2</f>
         <v>8</v>
       </c>
@@ -1172,7 +1165,7 @@
       <c r="E3" s="1">
         <v>2017.0</v>
       </c>
-      <c r="F3" s="6">
+      <c r="F3" s="5">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
@@ -1193,7 +1186,7 @@
       <c r="E4" s="1">
         <v>2012.0</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="5">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
@@ -1214,7 +1207,7 @@
       <c r="E5" s="1">
         <v>2021.0</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="5">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
@@ -1235,7 +1228,7 @@
       <c r="E6" s="1">
         <v>2021.0</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="5">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
@@ -1256,7 +1249,7 @@
       <c r="E7" s="1">
         <v>2017.0</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="5">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
@@ -1277,7 +1270,7 @@
       <c r="E8" s="1">
         <v>2017.0</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="5">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
@@ -1298,7 +1291,7 @@
       <c r="E9" s="1">
         <v>2018.0</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="5">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
@@ -1319,7 +1312,7 @@
       <c r="E10" s="1">
         <v>2023.0</v>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="5">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
@@ -1340,7 +1333,7 @@
       <c r="E11" s="1">
         <v>2012.0</v>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="5">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
@@ -1361,7 +1354,7 @@
       <c r="E12" s="1">
         <v>2012.0</v>
       </c>
-      <c r="F12" s="6">
+      <c r="F12" s="5">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
@@ -1382,7 +1375,7 @@
       <c r="E13" s="1">
         <v>2012.0</v>
       </c>
-      <c r="F13" s="6">
+      <c r="F13" s="5">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
@@ -1403,7 +1396,7 @@
       <c r="E14" s="1">
         <v>2017.0</v>
       </c>
-      <c r="F14" s="6">
+      <c r="F14" s="5">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
@@ -1424,7 +1417,7 @@
       <c r="E15" s="1">
         <v>2024.0</v>
       </c>
-      <c r="F15" s="6">
+      <c r="F15" s="5">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
@@ -1445,7 +1438,7 @@
       <c r="E16" s="1">
         <v>2017.0</v>
       </c>
-      <c r="F16" s="6">
+      <c r="F16" s="5">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
@@ -1466,7 +1459,7 @@
       <c r="E17" s="1">
         <v>2017.0</v>
       </c>
-      <c r="F17" s="6">
+      <c r="F17" s="5">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
@@ -1487,7 +1480,7 @@
       <c r="E18" s="1">
         <v>2018.0</v>
       </c>
-      <c r="F18" s="6">
+      <c r="F18" s="5">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
@@ -1508,7 +1501,7 @@
       <c r="E19" s="1">
         <v>2018.0</v>
       </c>
-      <c r="F19" s="6">
+      <c r="F19" s="5">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
@@ -1529,7 +1522,7 @@
       <c r="E20" s="1">
         <v>2018.0</v>
       </c>
-      <c r="F20" s="6">
+      <c r="F20" s="5">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
@@ -1550,7 +1543,7 @@
       <c r="E21" s="1">
         <v>2018.0</v>
       </c>
-      <c r="F21" s="6">
+      <c r="F21" s="5">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
@@ -1571,7 +1564,7 @@
       <c r="E22" s="1">
         <v>2012.0</v>
       </c>
-      <c r="F22" s="6">
+      <c r="F22" s="5">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
@@ -1592,7 +1585,7 @@
       <c r="E23" s="1">
         <v>2024.0</v>
       </c>
-      <c r="F23" s="6">
+      <c r="F23" s="5">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
@@ -1627,7 +1620,7 @@
       <c r="B2" s="1">
         <v>1.0</v>
       </c>
-      <c r="C2" s="6">
+      <c r="C2" s="5">
         <v>98749.0</v>
       </c>
     </row>
@@ -1638,7 +1631,7 @@
       <c r="B3" s="1">
         <v>1.0</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3" s="5">
         <v>98750.0</v>
       </c>
     </row>
@@ -1649,7 +1642,7 @@
       <c r="B4" s="1">
         <v>1.0</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="5">
         <v>98751.0</v>
       </c>
     </row>
@@ -1660,7 +1653,7 @@
       <c r="B5" s="1">
         <v>1.0</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="5">
         <v>98752.0</v>
       </c>
     </row>
@@ -1671,7 +1664,7 @@
       <c r="B6" s="1">
         <v>1.0</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="5">
         <v>98753.0</v>
       </c>
     </row>
@@ -1682,7 +1675,7 @@
       <c r="B7" s="1">
         <v>1.0</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="5">
         <v>98754.0</v>
       </c>
     </row>
@@ -1693,7 +1686,7 @@
       <c r="B8" s="1">
         <v>2.0</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="5">
         <v>98750.0</v>
       </c>
     </row>
@@ -1704,7 +1697,7 @@
       <c r="B9" s="1">
         <v>2.0</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="5">
         <v>98751.0</v>
       </c>
     </row>
@@ -1715,7 +1708,7 @@
       <c r="B10" s="1">
         <v>2.0</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="5">
         <v>98752.0</v>
       </c>
     </row>
@@ -1726,7 +1719,7 @@
       <c r="B11" s="1">
         <v>2.0</v>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="5">
         <v>98753.0</v>
       </c>
     </row>
@@ -1737,7 +1730,7 @@
       <c r="B12" s="1">
         <v>2.0</v>
       </c>
-      <c r="C12" s="6">
+      <c r="C12" s="5">
         <v>98754.0</v>
       </c>
     </row>
@@ -1748,7 +1741,7 @@
       <c r="B13" s="1">
         <v>3.0</v>
       </c>
-      <c r="C13" s="6">
+      <c r="C13" s="5">
         <v>98749.0</v>
       </c>
     </row>
@@ -1759,7 +1752,7 @@
       <c r="B14" s="1">
         <v>3.0</v>
       </c>
-      <c r="C14" s="6">
+      <c r="C14" s="5">
         <v>98750.0</v>
       </c>
     </row>
@@ -1770,7 +1763,7 @@
       <c r="B15" s="1">
         <v>3.0</v>
       </c>
-      <c r="C15" s="6">
+      <c r="C15" s="5">
         <v>98751.0</v>
       </c>
     </row>
@@ -1781,7 +1774,7 @@
       <c r="B16" s="1">
         <v>3.0</v>
       </c>
-      <c r="C16" s="6">
+      <c r="C16" s="5">
         <v>98752.0</v>
       </c>
     </row>
@@ -1792,7 +1785,7 @@
       <c r="B17" s="1">
         <v>3.0</v>
       </c>
-      <c r="C17" s="6">
+      <c r="C17" s="5">
         <v>98753.0</v>
       </c>
     </row>
@@ -1803,7 +1796,7 @@
       <c r="B18" s="1">
         <v>3.0</v>
       </c>
-      <c r="C18" s="6">
+      <c r="C18" s="5">
         <v>98754.0</v>
       </c>
     </row>
@@ -1814,7 +1807,7 @@
       <c r="B19" s="1">
         <v>4.0</v>
       </c>
-      <c r="C19" s="6">
+      <c r="C19" s="5">
         <v>98752.0</v>
       </c>
     </row>
@@ -1825,7 +1818,7 @@
       <c r="B20" s="1">
         <v>4.0</v>
       </c>
-      <c r="C20" s="6">
+      <c r="C20" s="5">
         <v>98753.0</v>
       </c>
     </row>
@@ -1836,7 +1829,7 @@
       <c r="B21" s="1">
         <v>5.0</v>
       </c>
-      <c r="C21" s="6">
+      <c r="C21" s="5">
         <v>98752.0</v>
       </c>
     </row>
@@ -1847,7 +1840,7 @@
       <c r="B22" s="1">
         <v>5.0</v>
       </c>
-      <c r="C22" s="6">
+      <c r="C22" s="5">
         <v>98753.0</v>
       </c>
     </row>
@@ -1858,7 +1851,7 @@
       <c r="B23" s="1">
         <v>6.0</v>
       </c>
-      <c r="C23" s="6">
+      <c r="C23" s="5">
         <v>98750.0</v>
       </c>
     </row>
@@ -1869,7 +1862,7 @@
       <c r="B24" s="1">
         <v>6.0</v>
       </c>
-      <c r="C24" s="6">
+      <c r="C24" s="5">
         <v>98751.0</v>
       </c>
     </row>
@@ -1880,7 +1873,7 @@
       <c r="B25" s="1">
         <v>7.0</v>
       </c>
-      <c r="C25" s="6">
+      <c r="C25" s="5">
         <v>98749.0</v>
       </c>
     </row>
@@ -1891,7 +1884,7 @@
       <c r="B26" s="1">
         <v>8.0</v>
       </c>
-      <c r="C26" s="6">
+      <c r="C26" s="5">
         <v>98750.0</v>
       </c>
     </row>
@@ -1902,7 +1895,7 @@
       <c r="B27" s="1">
         <v>8.0</v>
       </c>
-      <c r="C27" s="6">
+      <c r="C27" s="5">
         <v>98751.0</v>
       </c>
     </row>
@@ -1913,7 +1906,7 @@
       <c r="B28" s="1">
         <v>8.0</v>
       </c>
-      <c r="C28" s="6">
+      <c r="C28" s="5">
         <v>98752.0</v>
       </c>
     </row>
@@ -1924,7 +1917,7 @@
       <c r="B29" s="1">
         <v>8.0</v>
       </c>
-      <c r="C29" s="6">
+      <c r="C29" s="5">
         <v>98753.0</v>
       </c>
     </row>
@@ -1935,7 +1928,7 @@
       <c r="B30" s="1">
         <v>8.0</v>
       </c>
-      <c r="C30" s="6">
+      <c r="C30" s="5">
         <v>98754.0</v>
       </c>
     </row>
@@ -1946,7 +1939,7 @@
       <c r="B31" s="1">
         <v>9.0</v>
       </c>
-      <c r="C31" s="6">
+      <c r="C31" s="5">
         <v>98752.0</v>
       </c>
     </row>
@@ -1957,7 +1950,7 @@
       <c r="B32" s="1">
         <v>9.0</v>
       </c>
-      <c r="C32" s="6">
+      <c r="C32" s="5">
         <v>98753.0</v>
       </c>
     </row>
@@ -1968,7 +1961,7 @@
       <c r="B33" s="1">
         <v>9.0</v>
       </c>
-      <c r="C33" s="6">
+      <c r="C33" s="5">
         <v>98754.0</v>
       </c>
     </row>
@@ -1979,7 +1972,7 @@
       <c r="B34" s="1">
         <v>10.0</v>
       </c>
-      <c r="C34" s="8">
+      <c r="C34" s="7">
         <v>98746.0</v>
       </c>
     </row>
@@ -1990,7 +1983,7 @@
       <c r="B35" s="1">
         <v>10.0</v>
       </c>
-      <c r="C35" s="8">
+      <c r="C35" s="7">
         <v>98747.0</v>
       </c>
     </row>
@@ -2001,7 +1994,7 @@
       <c r="B36" s="1">
         <v>10.0</v>
       </c>
-      <c r="C36" s="8">
+      <c r="C36" s="7">
         <v>98750.0</v>
       </c>
     </row>
@@ -2012,7 +2005,7 @@
       <c r="B37" s="1">
         <v>10.0</v>
       </c>
-      <c r="C37" s="8">
+      <c r="C37" s="7">
         <v>98751.0</v>
       </c>
     </row>
@@ -2023,7 +2016,7 @@
       <c r="B38" s="1">
         <v>10.0</v>
       </c>
-      <c r="C38" s="8">
+      <c r="C38" s="7">
         <v>98752.0</v>
       </c>
     </row>
@@ -2034,7 +2027,7 @@
       <c r="B39" s="1">
         <v>10.0</v>
       </c>
-      <c r="C39" s="8">
+      <c r="C39" s="7">
         <v>98753.0</v>
       </c>
     </row>
@@ -2045,7 +2038,7 @@
       <c r="B40" s="1">
         <v>10.0</v>
       </c>
-      <c r="C40" s="8">
+      <c r="C40" s="7">
         <v>98754.0</v>
       </c>
     </row>
@@ -2056,7 +2049,7 @@
       <c r="B41" s="1">
         <v>11.0</v>
       </c>
-      <c r="C41" s="8">
+      <c r="C41" s="7">
         <v>98746.0</v>
       </c>
     </row>
@@ -2067,7 +2060,7 @@
       <c r="B42" s="1">
         <v>11.0</v>
       </c>
-      <c r="C42" s="8">
+      <c r="C42" s="7">
         <v>98747.0</v>
       </c>
     </row>
@@ -2078,7 +2071,7 @@
       <c r="B43" s="1">
         <v>11.0</v>
       </c>
-      <c r="C43" s="8">
+      <c r="C43" s="7">
         <v>98750.0</v>
       </c>
     </row>
@@ -2089,7 +2082,7 @@
       <c r="B44" s="1">
         <v>11.0</v>
       </c>
-      <c r="C44" s="8">
+      <c r="C44" s="7">
         <v>98751.0</v>
       </c>
     </row>
@@ -2100,7 +2093,7 @@
       <c r="B45" s="1">
         <v>11.0</v>
       </c>
-      <c r="C45" s="8">
+      <c r="C45" s="7">
         <v>98752.0</v>
       </c>
     </row>
@@ -2111,7 +2104,7 @@
       <c r="B46" s="1">
         <v>11.0</v>
       </c>
-      <c r="C46" s="8">
+      <c r="C46" s="7">
         <v>98753.0</v>
       </c>
     </row>
@@ -2122,7 +2115,7 @@
       <c r="B47" s="1">
         <v>11.0</v>
       </c>
-      <c r="C47" s="8">
+      <c r="C47" s="7">
         <v>98754.0</v>
       </c>
     </row>
@@ -2133,7 +2126,7 @@
       <c r="B48" s="1">
         <v>12.0</v>
       </c>
-      <c r="C48" s="8">
+      <c r="C48" s="7">
         <v>98746.0</v>
       </c>
     </row>
@@ -2144,7 +2137,7 @@
       <c r="B49" s="1">
         <v>12.0</v>
       </c>
-      <c r="C49" s="8">
+      <c r="C49" s="7">
         <v>98747.0</v>
       </c>
     </row>
@@ -2155,7 +2148,7 @@
       <c r="B50" s="1">
         <v>12.0</v>
       </c>
-      <c r="C50" s="8">
+      <c r="C50" s="7">
         <v>98750.0</v>
       </c>
     </row>
@@ -2166,7 +2159,7 @@
       <c r="B51" s="1">
         <v>12.0</v>
       </c>
-      <c r="C51" s="8">
+      <c r="C51" s="7">
         <v>98751.0</v>
       </c>
     </row>
@@ -2177,7 +2170,7 @@
       <c r="B52" s="1">
         <v>12.0</v>
       </c>
-      <c r="C52" s="8">
+      <c r="C52" s="7">
         <v>98752.0</v>
       </c>
     </row>
@@ -2188,7 +2181,7 @@
       <c r="B53" s="1">
         <v>12.0</v>
       </c>
-      <c r="C53" s="8">
+      <c r="C53" s="7">
         <v>98753.0</v>
       </c>
     </row>
@@ -2199,7 +2192,7 @@
       <c r="B54" s="1">
         <v>12.0</v>
       </c>
-      <c r="C54" s="8">
+      <c r="C54" s="7">
         <v>98754.0</v>
       </c>
     </row>
@@ -2210,7 +2203,7 @@
       <c r="B55" s="1">
         <v>13.0</v>
       </c>
-      <c r="C55" s="6">
+      <c r="C55" s="5">
         <v>98749.0</v>
       </c>
     </row>
@@ -2221,7 +2214,7 @@
       <c r="B56" s="1">
         <v>13.0</v>
       </c>
-      <c r="C56" s="6">
+      <c r="C56" s="5">
         <v>98750.0</v>
       </c>
     </row>
@@ -2232,7 +2225,7 @@
       <c r="B57" s="1">
         <v>13.0</v>
       </c>
-      <c r="C57" s="6">
+      <c r="C57" s="5">
         <v>98751.0</v>
       </c>
     </row>
@@ -2243,7 +2236,7 @@
       <c r="B58" s="1">
         <v>13.0</v>
       </c>
-      <c r="C58" s="6">
+      <c r="C58" s="5">
         <v>98752.0</v>
       </c>
     </row>
@@ -2254,7 +2247,7 @@
       <c r="B59" s="1">
         <v>13.0</v>
       </c>
-      <c r="C59" s="6">
+      <c r="C59" s="5">
         <v>98753.0</v>
       </c>
     </row>
@@ -2265,7 +2258,7 @@
       <c r="B60" s="1">
         <v>13.0</v>
       </c>
-      <c r="C60" s="6">
+      <c r="C60" s="5">
         <v>98754.0</v>
       </c>
     </row>
@@ -2276,7 +2269,7 @@
       <c r="B61" s="1">
         <v>14.0</v>
       </c>
-      <c r="C61" s="6">
+      <c r="C61" s="5">
         <v>98753.0</v>
       </c>
     </row>
@@ -2287,7 +2280,7 @@
       <c r="B62" s="1">
         <v>14.0</v>
       </c>
-      <c r="C62" s="6">
+      <c r="C62" s="5">
         <v>98754.0</v>
       </c>
     </row>
@@ -2298,7 +2291,7 @@
       <c r="B63" s="1">
         <v>15.0</v>
       </c>
-      <c r="C63" s="6">
+      <c r="C63" s="5">
         <v>98749.0</v>
       </c>
     </row>
@@ -2309,7 +2302,7 @@
       <c r="B64" s="1">
         <v>15.0</v>
       </c>
-      <c r="C64" s="6">
+      <c r="C64" s="5">
         <v>98750.0</v>
       </c>
     </row>
@@ -2320,7 +2313,7 @@
       <c r="B65" s="1">
         <v>15.0</v>
       </c>
-      <c r="C65" s="6">
+      <c r="C65" s="5">
         <v>98751.0</v>
       </c>
     </row>
@@ -2331,7 +2324,7 @@
       <c r="B66" s="1">
         <v>15.0</v>
       </c>
-      <c r="C66" s="6">
+      <c r="C66" s="5">
         <v>98752.0</v>
       </c>
     </row>
@@ -2342,7 +2335,7 @@
       <c r="B67" s="1">
         <v>15.0</v>
       </c>
-      <c r="C67" s="6">
+      <c r="C67" s="5">
         <v>98753.0</v>
       </c>
     </row>
@@ -2353,7 +2346,7 @@
       <c r="B68" s="1">
         <v>15.0</v>
       </c>
-      <c r="C68" s="6">
+      <c r="C68" s="5">
         <v>98754.0</v>
       </c>
     </row>
@@ -2364,7 +2357,7 @@
       <c r="B69" s="1">
         <v>16.0</v>
       </c>
-      <c r="C69" s="6">
+      <c r="C69" s="5">
         <v>98749.0</v>
       </c>
     </row>
@@ -2375,7 +2368,7 @@
       <c r="B70" s="1">
         <v>16.0</v>
       </c>
-      <c r="C70" s="6">
+      <c r="C70" s="5">
         <v>98750.0</v>
       </c>
     </row>
@@ -2386,7 +2379,7 @@
       <c r="B71" s="1">
         <v>16.0</v>
       </c>
-      <c r="C71" s="6">
+      <c r="C71" s="5">
         <v>98751.0</v>
       </c>
     </row>
@@ -2397,7 +2390,7 @@
       <c r="B72" s="1">
         <v>16.0</v>
       </c>
-      <c r="C72" s="6">
+      <c r="C72" s="5">
         <v>98752.0</v>
       </c>
     </row>
@@ -2408,7 +2401,7 @@
       <c r="B73" s="1">
         <v>16.0</v>
       </c>
-      <c r="C73" s="6">
+      <c r="C73" s="5">
         <v>98753.0</v>
       </c>
     </row>
@@ -2419,7 +2412,7 @@
       <c r="B74" s="1">
         <v>16.0</v>
       </c>
-      <c r="C74" s="6">
+      <c r="C74" s="5">
         <v>98754.0</v>
       </c>
     </row>
@@ -2430,7 +2423,7 @@
       <c r="B75" s="1">
         <v>17.0</v>
       </c>
-      <c r="C75" s="6">
+      <c r="C75" s="5">
         <v>98749.0</v>
       </c>
     </row>
@@ -2441,7 +2434,7 @@
       <c r="B76" s="1">
         <v>17.0</v>
       </c>
-      <c r="C76" s="6">
+      <c r="C76" s="5">
         <v>98750.0</v>
       </c>
     </row>
@@ -2452,7 +2445,7 @@
       <c r="B77" s="1">
         <v>17.0</v>
       </c>
-      <c r="C77" s="6">
+      <c r="C77" s="5">
         <v>98751.0</v>
       </c>
     </row>
@@ -2463,7 +2456,7 @@
       <c r="B78" s="1">
         <v>17.0</v>
       </c>
-      <c r="C78" s="6">
+      <c r="C78" s="5">
         <v>98752.0</v>
       </c>
     </row>
@@ -2474,7 +2467,7 @@
       <c r="B79" s="1">
         <v>17.0</v>
       </c>
-      <c r="C79" s="6">
+      <c r="C79" s="5">
         <v>98753.0</v>
       </c>
     </row>
@@ -2485,7 +2478,7 @@
       <c r="B80" s="1">
         <v>17.0</v>
       </c>
-      <c r="C80" s="6">
+      <c r="C80" s="5">
         <v>98754.0</v>
       </c>
     </row>
@@ -2496,7 +2489,7 @@
       <c r="B81" s="1">
         <v>18.0</v>
       </c>
-      <c r="C81" s="6">
+      <c r="C81" s="5">
         <v>98750.0</v>
       </c>
     </row>
@@ -2507,7 +2500,7 @@
       <c r="B82" s="1">
         <v>18.0</v>
       </c>
-      <c r="C82" s="6">
+      <c r="C82" s="5">
         <v>98751.0</v>
       </c>
     </row>
@@ -2518,7 +2511,7 @@
       <c r="B83" s="1">
         <v>18.0</v>
       </c>
-      <c r="C83" s="6">
+      <c r="C83" s="5">
         <v>98752.0</v>
       </c>
     </row>
@@ -2529,7 +2522,7 @@
       <c r="B84" s="1">
         <v>18.0</v>
       </c>
-      <c r="C84" s="6">
+      <c r="C84" s="5">
         <v>98753.0</v>
       </c>
     </row>
@@ -2540,7 +2533,7 @@
       <c r="B85" s="1">
         <v>18.0</v>
       </c>
-      <c r="C85" s="6">
+      <c r="C85" s="5">
         <v>98754.0</v>
       </c>
     </row>
@@ -2551,7 +2544,7 @@
       <c r="B86" s="1">
         <v>19.0</v>
       </c>
-      <c r="C86" s="6">
+      <c r="C86" s="5">
         <v>98751.0</v>
       </c>
     </row>
@@ -2562,7 +2555,7 @@
       <c r="B87" s="1">
         <v>20.0</v>
       </c>
-      <c r="C87" s="6">
+      <c r="C87" s="5">
         <v>98752.0</v>
       </c>
     </row>
@@ -2573,7 +2566,7 @@
       <c r="B88" s="1">
         <v>20.0</v>
       </c>
-      <c r="C88" s="6">
+      <c r="C88" s="5">
         <v>98753.0</v>
       </c>
     </row>
@@ -2584,7 +2577,7 @@
       <c r="B89" s="1">
         <v>20.0</v>
       </c>
-      <c r="C89" s="6">
+      <c r="C89" s="5">
         <v>98754.0</v>
       </c>
     </row>
@@ -2595,7 +2588,7 @@
       <c r="B90" s="1">
         <v>21.0</v>
       </c>
-      <c r="C90" s="8">
+      <c r="C90" s="7">
         <v>98746.0</v>
       </c>
     </row>
@@ -2606,7 +2599,7 @@
       <c r="B91" s="1">
         <v>21.0</v>
       </c>
-      <c r="C91" s="8">
+      <c r="C91" s="7">
         <v>98747.0</v>
       </c>
     </row>
@@ -2617,7 +2610,7 @@
       <c r="B92" s="1">
         <v>21.0</v>
       </c>
-      <c r="C92" s="8">
+      <c r="C92" s="7">
         <v>98750.0</v>
       </c>
     </row>
@@ -2628,7 +2621,7 @@
       <c r="B93" s="1">
         <v>21.0</v>
       </c>
-      <c r="C93" s="8">
+      <c r="C93" s="7">
         <v>98751.0</v>
       </c>
     </row>
@@ -2639,7 +2632,7 @@
       <c r="B94" s="1">
         <v>21.0</v>
       </c>
-      <c r="C94" s="8">
+      <c r="C94" s="7">
         <v>98752.0</v>
       </c>
     </row>
@@ -2650,7 +2643,7 @@
       <c r="B95" s="1">
         <v>21.0</v>
       </c>
-      <c r="C95" s="8">
+      <c r="C95" s="7">
         <v>98753.0</v>
       </c>
     </row>
@@ -2661,7 +2654,7 @@
       <c r="B96" s="1">
         <v>21.0</v>
       </c>
-      <c r="C96" s="8">
+      <c r="C96" s="7">
         <v>98754.0</v>
       </c>
     </row>
@@ -2672,7 +2665,7 @@
       <c r="B97" s="1">
         <v>22.0</v>
       </c>
-      <c r="C97" s="6">
+      <c r="C97" s="5">
         <v>98753.0</v>
       </c>
     </row>
@@ -2683,7 +2676,7 @@
       <c r="B98" s="1">
         <v>22.0</v>
       </c>
-      <c r="C98" s="6">
+      <c r="C98" s="5">
         <v>98754.0</v>
       </c>
     </row>

</xml_diff>